<commit_message>
fix: resolve import contract P0 conflicts
</commit_message>
<xml_diff>
--- a/deliverables/pm/excel_templates/02_variants_v1.0.xlsx
+++ b/deliverables/pm/excel_templates/02_variants_v1.0.xlsx
@@ -838,6 +838,11 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:D1"/>
+  <dataValidations count="1">
+    <dataValidation sqref="D2:D1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="整数无效" error="请输入符合范围的整数" type="whole" operator="greaterThanOrEqual">
+      <formula1>1</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>

</xml_diff>